<commit_message>
Fix daily delivery template evening border
</commit_message>
<xml_diff>
--- a/backend/src/data/delivery_note_templates/daily_delivery_note_reference.xlsx
+++ b/backend/src/data/delivery_note_templates/daily_delivery_note_reference.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-15" yWindow="-15" windowWidth="9600" windowHeight="11925" tabRatio="721" firstSheet="4" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="テンプレート" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="テンプレート" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="aaa">#REF!</definedName>
@@ -353,7 +353,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="86">
+  <borders count="104">
     <border>
       <left/>
       <right/>
@@ -1424,6 +1424,230 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
@@ -1436,7 +1660,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="365">
+  <cellXfs count="384">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2474,6 +2698,51 @@
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="83" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="86" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="87" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="88" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="89" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="90" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="91" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="94" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="97" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="97" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="97" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="99" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="100" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="101" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="102" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="102" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="103" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -3174,8 +3443,8 @@
       <c r="K16" s="330" t="n"/>
     </row>
     <row r="17" ht="23.25" customHeight="1" s="290">
-      <c r="A17" s="183" t="n"/>
-      <c r="B17" s="325" t="inlineStr">
+      <c r="A17" s="371" t="n"/>
+      <c r="B17" s="372" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
@@ -3195,8 +3464,8 @@
       <c r="K17" s="15" t="n"/>
     </row>
     <row r="18" ht="23.25" customHeight="1" s="290">
-      <c r="A18" s="302" t="n"/>
-      <c r="B18" s="327" t="n"/>
+      <c r="A18" s="373" t="n"/>
+      <c r="B18" s="374" t="n"/>
       <c r="C18" s="325" t="inlineStr">
         <is>
           <t>副①</t>
@@ -3212,47 +3481,40 @@
       <c r="K18" s="328" t="n"/>
     </row>
     <row r="19" ht="23.25" customHeight="1" s="290" thickBot="1">
-      <c r="A19" s="331" t="n"/>
-      <c r="B19" s="323" t="n"/>
-      <c r="C19" s="332" t="inlineStr">
+      <c r="A19" s="375" t="n"/>
+      <c r="B19" s="376" t="n"/>
+      <c r="C19" s="365" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D19" s="112" t="n"/>
-      <c r="E19" s="201" t="n"/>
-      <c r="F19" s="201" t="n"/>
-      <c r="G19" s="201" t="n"/>
-      <c r="H19" s="201" t="n"/>
-      <c r="I19" s="201" t="n"/>
-      <c r="J19" s="333" t="n"/>
-      <c r="K19" s="334" t="n"/>
+      <c r="D19" s="377" t="n"/>
+      <c r="E19" s="367" t="n"/>
+      <c r="F19" s="367" t="n"/>
+      <c r="G19" s="367" t="n"/>
+      <c r="H19" s="367" t="n"/>
+      <c r="I19" s="367" t="n"/>
+      <c r="J19" s="378" t="n"/>
+      <c r="K19" s="379" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1" s="290">
-      <c r="A20" s="37" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t>　</t>
-        </is>
-      </c>
+      <c r="A20" s="380" t="n"/>
+      <c r="B20" s="381" t="n"/>
+      <c r="C20" s="381" t="n"/>
+      <c r="D20" s="382" t="n"/>
+      <c r="E20" s="381" t="n"/>
+      <c r="F20" s="381" t="n"/>
+      <c r="G20" s="381" t="n"/>
+      <c r="H20" s="381" t="n"/>
+      <c r="I20" s="381" t="n"/>
+      <c r="J20" s="381" t="n"/>
+      <c r="K20" s="383" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1" s="290">
-      <c r="C27" s="37" t="inlineStr">
-        <is>
-          <t>v</t>
-        </is>
-      </c>
+      <c r="C27" s="37" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1" s="290">
-      <c r="K31" s="1" t="inlineStr">
-        <is>
-          <t>./</t>
-        </is>
-      </c>
+      <c r="K31" s="1" t="n"/>
     </row>
     <row r="38" ht="18" customFormat="1" customHeight="1" s="28">
       <c r="A38" s="37" t="n"/>
@@ -3263,8 +3525,8 @@
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="J8:K11"/>
+    <mergeCell ref="B17:B19"/>
     <mergeCell ref="A12:A16"/>
-    <mergeCell ref="B17:B19"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="D8:D11"/>
     <mergeCell ref="B12:B13"/>

</xml_diff>

<commit_message>
Remove extra border from delivery template
</commit_message>
<xml_diff>
--- a/backend/src/data/delivery_note_templates/daily_delivery_note_reference.xlsx
+++ b/backend/src/data/delivery_note_templates/daily_delivery_note_reference.xlsx
@@ -353,7 +353,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="104">
+  <borders count="105">
     <border>
       <left/>
       <right/>
@@ -1648,6 +1648,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
@@ -1660,7 +1671,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="384">
+  <cellXfs count="387">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2743,6 +2754,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="103" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="93" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="96" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="104" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -3498,17 +3516,17 @@
       <c r="K19" s="379" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1" s="290">
-      <c r="A20" s="380" t="n"/>
-      <c r="B20" s="381" t="n"/>
-      <c r="C20" s="381" t="n"/>
-      <c r="D20" s="382" t="n"/>
-      <c r="E20" s="381" t="n"/>
-      <c r="F20" s="381" t="n"/>
-      <c r="G20" s="381" t="n"/>
-      <c r="H20" s="381" t="n"/>
-      <c r="I20" s="381" t="n"/>
-      <c r="J20" s="381" t="n"/>
-      <c r="K20" s="383" t="n"/>
+      <c r="A20" s="384" t="n"/>
+      <c r="B20" s="374" t="n"/>
+      <c r="C20" s="374" t="n"/>
+      <c r="D20" s="385" t="n"/>
+      <c r="E20" s="374" t="n"/>
+      <c r="F20" s="374" t="n"/>
+      <c r="G20" s="374" t="n"/>
+      <c r="H20" s="374" t="n"/>
+      <c r="I20" s="374" t="n"/>
+      <c r="J20" s="374" t="n"/>
+      <c r="K20" s="386" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1" s="290">
       <c r="C27" s="37" t="n"/>

</xml_diff>